<commit_message>
Add reviewed period payroll, starter proration and bonus inputs
</commit_message>
<xml_diff>
--- a/public/payroll-review.xlsx
+++ b/public/payroll-review.xlsx
@@ -13,9 +13,11 @@
     <sheet name="Calculation" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Reference" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Sources" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Period review" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Calculation!$A$1:$AA$16</definedName>
+    <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">'Period review'!$A$1:$Y$7</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -27,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="140">
   <si>
     <t xml:space="preserve">Nigeria 2026 payroll calculation review</t>
   </si>
@@ -41,7 +43,7 @@
     <t xml:space="preserve">Scope</t>
   </si>
   <si>
-    <t xml:space="preserve">Fixed, recurring monthly Nigerian employment pay; 2026 periods only.</t>
+    <t xml:space="preserve">Recurring monthly earnings plus reviewed period adjustments; Nigeria 2026 only.</t>
   </si>
   <si>
     <t xml:space="preserve">Instructions</t>
@@ -86,10 +88,16 @@
     <t xml:space="preserve">ECS default 1% gross. ITF is disabled until applicability is confirmed; normally 1% annual payroll for eligible employers.</t>
   </si>
   <si>
+    <t xml:space="preserve">Period adjustments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calendar-day starters, bonuses and one-off deductions. Period review sheet uses supplied reviewed PAYE, not a cumulative tax estimate. NHIS and recurring after-tax deductions are not prorated.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Not supported</t>
   </si>
   <si>
-    <t xml:space="preserve">Bonuses, variable pay, arrears, cumulative/YTD PAYE adjustments, mid-month prorating, foreign currency or nonresident cases.</t>
+    <t xml:space="preserve">Automatic cumulative/YTD PAYE, arrears, leaver calculations, unpaid absence, foreign currency or nonresident cases.</t>
   </si>
   <si>
     <t xml:space="preserve">Sources</t>
@@ -384,6 +392,63 @@
   </si>
   <si>
     <t xml:space="preserve">Eligibility and 1% annual payroll contribution.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calendar days</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paid days</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Basic monthly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Housing monthly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transport monthly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other monthly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bonus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pensionable bonus BHT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reviewed PAYE INPUT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NHIS fixed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recurring deductions fixed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One-off deduction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Net</t>
+  </si>
+  <si>
+    <t xml:space="preserve">October starter and bonus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Starter pensionable bonus NHF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">February half month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Full month pensionable bonus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partial minimum wage explicit zero</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Component rounding</t>
   </si>
 </sst>
 </file>
@@ -500,7 +565,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -534,6 +599,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -660,6 +729,10 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
@@ -843,7 +916,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
@@ -966,6 +1039,14 @@
       </c>
       <c r="B15" s="2" t="s">
         <v>28</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -993,15 +1074,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B2" s="3" t="n">
         <v>0.08</v>
@@ -1009,7 +1090,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B3" s="3" t="n">
         <v>0.1</v>
@@ -1017,7 +1098,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B4" s="3" t="n">
         <v>0.025</v>
@@ -1025,15 +1106,15 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B6" s="3" t="n">
         <v>0.2</v>
@@ -1041,7 +1122,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B7" s="4" t="n">
         <v>500000</v>
@@ -1057,7 +1138,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B9" s="3" t="n">
         <v>0.01</v>
@@ -1065,7 +1146,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B10" s="3" t="n">
         <v>0</v>
@@ -1073,10 +1154,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -1104,85 +1185,85 @@
   <sheetData>
     <row r="1" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>9</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O1" s="1" t="s">
         <v>11</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1214,10 +1295,10 @@
         <v>0</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="L2" s="7" t="n">
         <f aca="false">SUM(B2:E2)</f>
@@ -1284,7 +1365,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B3" s="5" t="n">
         <v>70000.01</v>
@@ -1311,10 +1392,10 @@
         <v>0</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="L3" s="7" t="n">
         <f aca="false">SUM(B3:E3)</f>
@@ -1381,7 +1462,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B4" s="5" t="n">
         <v>200000</v>
@@ -1408,10 +1489,10 @@
         <v>0</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="L4" s="7" t="n">
         <f aca="false">SUM(B4:E4)</f>
@@ -1478,7 +1559,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B5" s="5" t="n">
         <v>250000</v>
@@ -1505,10 +1586,10 @@
         <v>0</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="L5" s="7" t="n">
         <f aca="false">SUM(B5:E5)</f>
@@ -1575,7 +1656,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B6" s="5" t="n">
         <v>1000000</v>
@@ -1602,10 +1683,10 @@
         <v>0</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="L6" s="7" t="n">
         <f aca="false">SUM(B6:E6)</f>
@@ -1672,7 +1753,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B7" s="5" t="n">
         <v>2083333.33</v>
@@ -1699,10 +1780,10 @@
         <v>0</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="L7" s="7" t="n">
         <f aca="false">SUM(B7:E7)</f>
@@ -1769,7 +1850,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B8" s="5" t="n">
         <v>4166666.67</v>
@@ -1796,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="L8" s="7" t="n">
         <f aca="false">SUM(B8:E8)</f>
@@ -1866,7 +1947,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B9" s="5" t="n">
         <v>5000000</v>
@@ -1893,10 +1974,10 @@
         <v>0</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="L9" s="7" t="n">
         <f aca="false">SUM(B9:E9)</f>
@@ -1963,7 +2044,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B10" s="5" t="n">
         <v>200000</v>
@@ -1990,10 +2071,10 @@
         <v>0</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="L10" s="7" t="n">
         <f aca="false">SUM(B10:E10)</f>
@@ -2060,7 +2141,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B11" s="5" t="n">
         <v>350000</v>
@@ -2087,10 +2168,10 @@
         <v>0</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="L11" s="7" t="n">
         <f aca="false">SUM(B11:E11)</f>
@@ -2157,7 +2238,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B12" s="5" t="n">
         <v>250000</v>
@@ -2184,10 +2265,10 @@
         <v>0</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="K12" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="L12" s="7" t="n">
         <f aca="false">SUM(B12:E12)</f>
@@ -2254,7 +2335,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B13" s="5" t="n">
         <v>200000</v>
@@ -2281,10 +2362,10 @@
         <v>0</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="L13" s="7" t="n">
         <f aca="false">SUM(B13:E13)</f>
@@ -2351,7 +2432,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B14" s="5" t="n">
         <v>200000</v>
@@ -2378,10 +2459,10 @@
         <v>120000</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="K14" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="L14" s="7" t="n">
         <f aca="false">SUM(B14:E14)</f>
@@ -2448,7 +2529,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B15" s="5" t="n">
         <v>123456.78</v>
@@ -2475,10 +2556,10 @@
         <v>0</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="L15" s="7" t="n">
         <f aca="false">SUM(B15:E15)</f>
@@ -2545,7 +2626,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B16" s="5" t="n">
         <v>100000</v>
@@ -2572,10 +2653,10 @@
         <v>1200000</v>
       </c>
       <c r="J16" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="K16" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="L16" s="7" t="n">
         <f aca="false">SUM(B16:E16)</f>
@@ -2673,37 +2754,37 @@
   <sheetData>
     <row r="1" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2743,7 +2824,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B3" s="0" t="n">
         <v>70000.01</v>
@@ -2778,7 +2859,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B4" s="0" t="n">
         <v>200000</v>
@@ -2813,7 +2894,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B5" s="0" t="n">
         <v>250000</v>
@@ -2848,7 +2929,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B6" s="0" t="n">
         <v>1000000</v>
@@ -2883,7 +2964,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B7" s="0" t="n">
         <v>2083333.33</v>
@@ -2918,7 +2999,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B8" s="0" t="n">
         <v>4166666.67</v>
@@ -2953,7 +3034,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B9" s="0" t="n">
         <v>5000000</v>
@@ -2988,7 +3069,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B10" s="0" t="n">
         <v>350000</v>
@@ -3023,7 +3104,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B11" s="0" t="n">
         <v>350000</v>
@@ -3058,7 +3139,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B12" s="0" t="n">
         <v>250000</v>
@@ -3093,7 +3174,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B13" s="0" t="n">
         <v>350000</v>
@@ -3128,7 +3209,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B14" s="0" t="n">
         <v>200000</v>
@@ -3163,7 +3244,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B15" s="0" t="n">
         <v>150370.35</v>
@@ -3198,7 +3279,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B16" s="0" t="n">
         <v>100000</v>
@@ -3257,101 +3338,101 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
   </sheetData>
@@ -3373,4 +3454,622 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:Y7"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="2" style="0" width="23"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>134</v>
+      </c>
+      <c r="B2" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="C2" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="D2" s="9" t="n">
+        <v>310000</v>
+      </c>
+      <c r="E2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="9" t="n">
+        <v>50000</v>
+      </c>
+      <c r="I2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="9" t="n">
+        <v>12000</v>
+      </c>
+      <c r="K2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" s="9" t="n">
+        <v>5000</v>
+      </c>
+      <c r="N2" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="O2" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="P2" s="4" t="n">
+        <f aca="false">ROUND(D2*C2/B2,2)+ROUND(E2*C2/B2,2)+ROUND(F2*C2/B2,2)+ROUND(G2*C2/B2,2)+H2</f>
+        <v>210000</v>
+      </c>
+      <c r="Q2" s="4" t="n">
+        <f aca="false">IF(N2="Yes",ROUND(IF(Settings!$B$11="gross",P2,ROUND(D2*C2/B2,2)+ROUND(E2*C2/B2,2)+ROUND(F2*C2/B2,2)+I2)*Settings!$B$2,2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="R2" s="4" t="n">
+        <f aca="false">IF(N2="Yes",ROUND(IF(Settings!$B$11="gross",P2,ROUND(D2*C2/B2,2)+ROUND(E2*C2/B2,2)+ROUND(F2*C2/B2,2)+I2)*Settings!$B$3,2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="S2" s="4" t="n">
+        <f aca="false">IF(O2="Yes",ROUND(IF(Settings!$B$5="gross",P2,ROUND(D2*C2/B2,2))*Settings!$B$4,2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="T2" s="4" t="n">
+        <f aca="false">SUM(J2:M2)+Q2+S2</f>
+        <v>17000</v>
+      </c>
+      <c r="U2" s="4" t="n">
+        <f aca="false">P2-T2</f>
+        <v>193000</v>
+      </c>
+      <c r="V2" s="4" t="n">
+        <f aca="false">ROUND(P2*Settings!$B$9,2)</f>
+        <v>2100</v>
+      </c>
+      <c r="W2" s="4" t="n">
+        <f aca="false">ROUND(P2*Settings!$B$10,2)</f>
+        <v>0</v>
+      </c>
+      <c r="X2" s="4" t="n">
+        <v>193000</v>
+      </c>
+      <c r="Y2" s="4" t="n">
+        <f aca="false">U2-X2</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
+        <v>135</v>
+      </c>
+      <c r="B3" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="C3" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="D3" s="9" t="n">
+        <v>310000</v>
+      </c>
+      <c r="E3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="9" t="n">
+        <v>50000</v>
+      </c>
+      <c r="I3" s="9" t="n">
+        <v>20000</v>
+      </c>
+      <c r="J3" s="9" t="n">
+        <v>8000</v>
+      </c>
+      <c r="K3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="9" t="n">
+        <v>5000</v>
+      </c>
+      <c r="N3" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="O3" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="P3" s="4" t="n">
+        <f aca="false">ROUND(D3*C3/B3,2)+ROUND(E3*C3/B3,2)+ROUND(F3*C3/B3,2)+ROUND(G3*C3/B3,2)+H3</f>
+        <v>210000</v>
+      </c>
+      <c r="Q3" s="4" t="n">
+        <f aca="false">IF(N3="Yes",ROUND(IF(Settings!$B$11="gross",P3,ROUND(D3*C3/B3,2)+ROUND(E3*C3/B3,2)+ROUND(F3*C3/B3,2)+I3)*Settings!$B$2,2),0)</f>
+        <v>14400</v>
+      </c>
+      <c r="R3" s="4" t="n">
+        <f aca="false">IF(N3="Yes",ROUND(IF(Settings!$B$11="gross",P3,ROUND(D3*C3/B3,2)+ROUND(E3*C3/B3,2)+ROUND(F3*C3/B3,2)+I3)*Settings!$B$3,2),0)</f>
+        <v>18000</v>
+      </c>
+      <c r="S3" s="4" t="n">
+        <f aca="false">IF(O3="Yes",ROUND(IF(Settings!$B$5="gross",P3,ROUND(D3*C3/B3,2))*Settings!$B$4,2),0)</f>
+        <v>4000</v>
+      </c>
+      <c r="T3" s="4" t="n">
+        <f aca="false">SUM(J3:M3)+Q3+S3</f>
+        <v>31400</v>
+      </c>
+      <c r="U3" s="4" t="n">
+        <f aca="false">P3-T3</f>
+        <v>178600</v>
+      </c>
+      <c r="V3" s="4" t="n">
+        <f aca="false">ROUND(P3*Settings!$B$9,2)</f>
+        <v>2100</v>
+      </c>
+      <c r="W3" s="4" t="n">
+        <f aca="false">ROUND(P3*Settings!$B$10,2)</f>
+        <v>0</v>
+      </c>
+      <c r="X3" s="4" t="n">
+        <v>178600</v>
+      </c>
+      <c r="Y3" s="4" t="n">
+        <f aca="false">U3-X3</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="s">
+        <v>136</v>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="D4" s="9" t="n">
+        <v>200000</v>
+      </c>
+      <c r="E4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="9" t="n">
+        <v>3000</v>
+      </c>
+      <c r="K4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="O4" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <f aca="false">ROUND(D4*C4/B4,2)+ROUND(E4*C4/B4,2)+ROUND(F4*C4/B4,2)+ROUND(G4*C4/B4,2)+H4</f>
+        <v>100000</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <f aca="false">IF(N4="Yes",ROUND(IF(Settings!$B$11="gross",P4,ROUND(D4*C4/B4,2)+ROUND(E4*C4/B4,2)+ROUND(F4*C4/B4,2)+I4)*Settings!$B$2,2),0)</f>
+        <v>8000</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <f aca="false">IF(N4="Yes",ROUND(IF(Settings!$B$11="gross",P4,ROUND(D4*C4/B4,2)+ROUND(E4*C4/B4,2)+ROUND(F4*C4/B4,2)+I4)*Settings!$B$3,2),0)</f>
+        <v>10000</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <f aca="false">IF(O4="Yes",ROUND(IF(Settings!$B$5="gross",P4,ROUND(D4*C4/B4,2))*Settings!$B$4,2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="T4" s="4" t="n">
+        <f aca="false">SUM(J4:M4)+Q4+S4</f>
+        <v>11000</v>
+      </c>
+      <c r="U4" s="4" t="n">
+        <f aca="false">P4-T4</f>
+        <v>89000</v>
+      </c>
+      <c r="V4" s="4" t="n">
+        <f aca="false">ROUND(P4*Settings!$B$9,2)</f>
+        <v>1000</v>
+      </c>
+      <c r="W4" s="4" t="n">
+        <f aca="false">ROUND(P4*Settings!$B$10,2)</f>
+        <v>0</v>
+      </c>
+      <c r="X4" s="4" t="n">
+        <v>89000</v>
+      </c>
+      <c r="Y4" s="4" t="n">
+        <f aca="false">U4-X4</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
+        <v>137</v>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>200000</v>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>100000</v>
+      </c>
+      <c r="I5" s="9" t="n">
+        <v>100000</v>
+      </c>
+      <c r="J5" s="9" t="n">
+        <v>25000</v>
+      </c>
+      <c r="K5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="O5" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="P5" s="4" t="n">
+        <f aca="false">ROUND(D5*C5/B5,2)+ROUND(E5*C5/B5,2)+ROUND(F5*C5/B5,2)+ROUND(G5*C5/B5,2)+H5</f>
+        <v>300000</v>
+      </c>
+      <c r="Q5" s="4" t="n">
+        <f aca="false">IF(N5="Yes",ROUND(IF(Settings!$B$11="gross",P5,ROUND(D5*C5/B5,2)+ROUND(E5*C5/B5,2)+ROUND(F5*C5/B5,2)+I5)*Settings!$B$2,2),0)</f>
+        <v>24000</v>
+      </c>
+      <c r="R5" s="4" t="n">
+        <f aca="false">IF(N5="Yes",ROUND(IF(Settings!$B$11="gross",P5,ROUND(D5*C5/B5,2)+ROUND(E5*C5/B5,2)+ROUND(F5*C5/B5,2)+I5)*Settings!$B$3,2),0)</f>
+        <v>30000</v>
+      </c>
+      <c r="S5" s="4" t="n">
+        <f aca="false">IF(O5="Yes",ROUND(IF(Settings!$B$5="gross",P5,ROUND(D5*C5/B5,2))*Settings!$B$4,2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="T5" s="4" t="n">
+        <f aca="false">SUM(J5:M5)+Q5+S5</f>
+        <v>49000</v>
+      </c>
+      <c r="U5" s="4" t="n">
+        <f aca="false">P5-T5</f>
+        <v>251000</v>
+      </c>
+      <c r="V5" s="4" t="n">
+        <f aca="false">ROUND(P5*Settings!$B$9,2)</f>
+        <v>3000</v>
+      </c>
+      <c r="W5" s="4" t="n">
+        <f aca="false">ROUND(P5*Settings!$B$10,2)</f>
+        <v>0</v>
+      </c>
+      <c r="X5" s="4" t="n">
+        <v>251000</v>
+      </c>
+      <c r="Y5" s="4" t="n">
+        <f aca="false">U5-X5</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="s">
+        <v>138</v>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>70000</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="O6" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <f aca="false">ROUND(D6*C6/B6,2)+ROUND(E6*C6/B6,2)+ROUND(F6*C6/B6,2)+ROUND(G6*C6/B6,2)+H6</f>
+        <v>2258.06</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <f aca="false">IF(N6="Yes",ROUND(IF(Settings!$B$11="gross",P6,ROUND(D6*C6/B6,2)+ROUND(E6*C6/B6,2)+ROUND(F6*C6/B6,2)+I6)*Settings!$B$2,2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <f aca="false">IF(N6="Yes",ROUND(IF(Settings!$B$11="gross",P6,ROUND(D6*C6/B6,2)+ROUND(E6*C6/B6,2)+ROUND(F6*C6/B6,2)+I6)*Settings!$B$3,2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <f aca="false">IF(O6="Yes",ROUND(IF(Settings!$B$5="gross",P6,ROUND(D6*C6/B6,2))*Settings!$B$4,2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="T6" s="4" t="n">
+        <f aca="false">SUM(J6:M6)+Q6+S6</f>
+        <v>0</v>
+      </c>
+      <c r="U6" s="4" t="n">
+        <f aca="false">P6-T6</f>
+        <v>2258.06</v>
+      </c>
+      <c r="V6" s="4" t="n">
+        <f aca="false">ROUND(P6*Settings!$B$9,2)</f>
+        <v>22.58</v>
+      </c>
+      <c r="W6" s="4" t="n">
+        <f aca="false">ROUND(P6*Settings!$B$10,2)</f>
+        <v>0</v>
+      </c>
+      <c r="X6" s="4" t="n">
+        <v>2258.06</v>
+      </c>
+      <c r="Y6" s="4" t="n">
+        <f aca="false">U6-X6</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>123456.78</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>23456.79</v>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>3456.78</v>
+      </c>
+      <c r="G7" s="9" t="n">
+        <v>111.11</v>
+      </c>
+      <c r="H7" s="9" t="n">
+        <v>500.01</v>
+      </c>
+      <c r="I7" s="9" t="n">
+        <v>100.01</v>
+      </c>
+      <c r="J7" s="9" t="n">
+        <v>1500.01</v>
+      </c>
+      <c r="K7" s="9" t="n">
+        <v>123.45</v>
+      </c>
+      <c r="L7" s="9" t="n">
+        <v>11.11</v>
+      </c>
+      <c r="M7" s="9" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="N7" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="O7" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="P7" s="4" t="n">
+        <f aca="false">ROUND(D7*C7/B7,2)+ROUND(E7*C7/B7,2)+ROUND(F7*C7/B7,2)+ROUND(G7*C7/B7,2)+H7</f>
+        <v>73313.62</v>
+      </c>
+      <c r="Q7" s="4" t="n">
+        <f aca="false">IF(N7="Yes",ROUND(IF(Settings!$B$11="gross",P7,ROUND(D7*C7/B7,2)+ROUND(E7*C7/B7,2)+ROUND(F7*C7/B7,2)+I7)*Settings!$B$2,2),0)</f>
+        <v>5828.79</v>
+      </c>
+      <c r="R7" s="4" t="n">
+        <f aca="false">IF(N7="Yes",ROUND(IF(Settings!$B$11="gross",P7,ROUND(D7*C7/B7,2)+ROUND(E7*C7/B7,2)+ROUND(F7*C7/B7,2)+I7)*Settings!$B$3,2),0)</f>
+        <v>7285.99</v>
+      </c>
+      <c r="S7" s="4" t="n">
+        <f aca="false">IF(O7="Yes",ROUND(IF(Settings!$B$5="gross",P7,ROUND(D7*C7/B7,2))*Settings!$B$4,2),0)</f>
+        <v>1493.43</v>
+      </c>
+      <c r="T7" s="4" t="n">
+        <f aca="false">SUM(J7:M7)+Q7+S7</f>
+        <v>8959.01</v>
+      </c>
+      <c r="U7" s="4" t="n">
+        <f aca="false">P7-T7</f>
+        <v>64354.61</v>
+      </c>
+      <c r="V7" s="4" t="n">
+        <f aca="false">ROUND(P7*Settings!$B$9,2)</f>
+        <v>733.14</v>
+      </c>
+      <c r="W7" s="4" t="n">
+        <f aca="false">ROUND(P7*Settings!$B$10,2)</f>
+        <v>0</v>
+      </c>
+      <c r="X7" s="4" t="n">
+        <v>64354.61</v>
+      </c>
+      <c r="Y7" s="4" t="n">
+        <f aca="false">U7-X7</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:Y7"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add reviewed opening balances, YTD payroll reconciliation and review records
</commit_message>
<xml_diff>
--- a/public/payroll-review.xlsx
+++ b/public/payroll-review.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Reference" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Sources" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Period review" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="YTD reconciliation" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Calculation!$A$1:$AA$16</definedName>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="168">
   <si>
     <t xml:space="preserve">Nigeria 2026 payroll calculation review</t>
   </si>
@@ -112,6 +113,12 @@
     <t xml:space="preserve">Reference sheet uses Python Decimal with cumulative thresholds; Calculation uses editable Excel marginal-band formulas.</t>
   </si>
   <si>
+    <t xml:space="preserve">YTD reconciliation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Separate sheet verifies opening + released totals and draft exclusion. This does not compute cumulative PAYE liability.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Signoff</t>
   </si>
   <si>
@@ -449,6 +456,84 @@
   </si>
   <si>
     <t xml:space="preserve">Component rounding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scenario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opening gross</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opening PAYE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opening employee pension</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opening other employee deductions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Released gross</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Released PAYE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Released employee pension</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Released other employee deductions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Draft gross EXCLUDED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YTD gross</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YTD PAYE withheld</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YTD deductions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YTD net</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Expected gross</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gross delta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opening only</t>
+  </si>
+  <si>
+    <t xml:space="preserve">October released</t>
+  </si>
+  <si>
+    <t xml:space="preserve">November draft excluded</t>
+  </si>
+  <si>
+    <t xml:space="preserve">October and November released</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Basis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opening balances cover January through a reviewed cutoff; only Approved/Paid payroll is included afterwards. Drafts do not affect totals.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tax status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PAYE is withheld, not confirmed remittance. This sheet does not calculate cumulative tax liability or verify external accountant identity.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evidence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opening references and change history are company-admin only. Released payroll review records include a calculation SHA-256 fingerprint.</t>
   </si>
 </sst>
 </file>
@@ -916,7 +1001,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
@@ -1047,6 +1132,14 @@
       </c>
       <c r="B16" s="2" t="s">
         <v>30</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -1074,15 +1167,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B2" s="3" t="n">
         <v>0.08</v>
@@ -1090,7 +1183,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B3" s="3" t="n">
         <v>0.1</v>
@@ -1098,7 +1191,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B4" s="3" t="n">
         <v>0.025</v>
@@ -1106,15 +1199,15 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B6" s="3" t="n">
         <v>0.2</v>
@@ -1122,7 +1215,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B7" s="4" t="n">
         <v>500000</v>
@@ -1138,7 +1231,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B9" s="3" t="n">
         <v>0.01</v>
@@ -1146,7 +1239,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B10" s="3" t="n">
         <v>0</v>
@@ -1154,10 +1247,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -1185,85 +1278,85 @@
   <sheetData>
     <row r="1" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>9</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="O1" s="1" t="s">
         <v>11</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1295,10 +1388,10 @@
         <v>0</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L2" s="7" t="n">
         <f aca="false">SUM(B2:E2)</f>
@@ -1365,7 +1458,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B3" s="5" t="n">
         <v>70000.01</v>
@@ -1392,10 +1485,10 @@
         <v>0</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L3" s="7" t="n">
         <f aca="false">SUM(B3:E3)</f>
@@ -1462,7 +1555,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B4" s="5" t="n">
         <v>200000</v>
@@ -1489,10 +1582,10 @@
         <v>0</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L4" s="7" t="n">
         <f aca="false">SUM(B4:E4)</f>
@@ -1559,7 +1652,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B5" s="5" t="n">
         <v>250000</v>
@@ -1586,10 +1679,10 @@
         <v>0</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L5" s="7" t="n">
         <f aca="false">SUM(B5:E5)</f>
@@ -1656,7 +1749,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B6" s="5" t="n">
         <v>1000000</v>
@@ -1683,10 +1776,10 @@
         <v>0</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L6" s="7" t="n">
         <f aca="false">SUM(B6:E6)</f>
@@ -1753,7 +1846,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B7" s="5" t="n">
         <v>2083333.33</v>
@@ -1780,10 +1873,10 @@
         <v>0</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L7" s="7" t="n">
         <f aca="false">SUM(B7:E7)</f>
@@ -1850,7 +1943,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B8" s="5" t="n">
         <v>4166666.67</v>
@@ -1877,10 +1970,10 @@
         <v>0</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L8" s="7" t="n">
         <f aca="false">SUM(B8:E8)</f>
@@ -1947,7 +2040,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B9" s="5" t="n">
         <v>5000000</v>
@@ -1974,10 +2067,10 @@
         <v>0</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L9" s="7" t="n">
         <f aca="false">SUM(B9:E9)</f>
@@ -2044,7 +2137,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B10" s="5" t="n">
         <v>200000</v>
@@ -2071,10 +2164,10 @@
         <v>0</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L10" s="7" t="n">
         <f aca="false">SUM(B10:E10)</f>
@@ -2141,7 +2234,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B11" s="5" t="n">
         <v>350000</v>
@@ -2168,10 +2261,10 @@
         <v>0</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L11" s="7" t="n">
         <f aca="false">SUM(B11:E11)</f>
@@ -2238,7 +2331,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B12" s="5" t="n">
         <v>250000</v>
@@ -2265,10 +2358,10 @@
         <v>0</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K12" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L12" s="7" t="n">
         <f aca="false">SUM(B12:E12)</f>
@@ -2335,7 +2428,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B13" s="5" t="n">
         <v>200000</v>
@@ -2362,10 +2455,10 @@
         <v>0</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L13" s="7" t="n">
         <f aca="false">SUM(B13:E13)</f>
@@ -2432,7 +2525,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B14" s="5" t="n">
         <v>200000</v>
@@ -2459,10 +2552,10 @@
         <v>120000</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K14" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L14" s="7" t="n">
         <f aca="false">SUM(B14:E14)</f>
@@ -2529,7 +2622,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B15" s="5" t="n">
         <v>123456.78</v>
@@ -2556,10 +2649,10 @@
         <v>0</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L15" s="7" t="n">
         <f aca="false">SUM(B15:E15)</f>
@@ -2626,7 +2719,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B16" s="5" t="n">
         <v>100000</v>
@@ -2653,10 +2746,10 @@
         <v>1200000</v>
       </c>
       <c r="J16" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="K16" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L16" s="7" t="n">
         <f aca="false">SUM(B16:E16)</f>
@@ -2754,37 +2847,37 @@
   <sheetData>
     <row r="1" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2824,7 +2917,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B3" s="0" t="n">
         <v>70000.01</v>
@@ -2859,7 +2952,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B4" s="0" t="n">
         <v>200000</v>
@@ -2894,7 +2987,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B5" s="0" t="n">
         <v>250000</v>
@@ -2929,7 +3022,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B6" s="0" t="n">
         <v>1000000</v>
@@ -2964,7 +3057,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B7" s="0" t="n">
         <v>2083333.33</v>
@@ -2999,7 +3092,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B8" s="0" t="n">
         <v>4166666.67</v>
@@ -3034,7 +3127,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B9" s="0" t="n">
         <v>5000000</v>
@@ -3069,7 +3162,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B10" s="0" t="n">
         <v>350000</v>
@@ -3104,7 +3197,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B11" s="0" t="n">
         <v>350000</v>
@@ -3139,7 +3232,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B12" s="0" t="n">
         <v>250000</v>
@@ -3174,7 +3267,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B13" s="0" t="n">
         <v>350000</v>
@@ -3209,7 +3302,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B14" s="0" t="n">
         <v>200000</v>
@@ -3244,7 +3337,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B15" s="0" t="n">
         <v>150370.35</v>
@@ -3279,7 +3372,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B16" s="0" t="n">
         <v>100000</v>
@@ -3338,101 +3431,101 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
   </sheetData>
@@ -3470,84 +3563,84 @@
   <sheetData>
     <row r="1" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="S1" s="1" t="s">
         <v>11</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B2" s="6" t="n">
         <v>31</v>
@@ -3586,10 +3679,10 @@
         <v>5000</v>
       </c>
       <c r="N2" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="O2" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="P2" s="4" t="n">
         <f aca="false">ROUND(D2*C2/B2,2)+ROUND(E2*C2/B2,2)+ROUND(F2*C2/B2,2)+ROUND(G2*C2/B2,2)+H2</f>
@@ -3633,7 +3726,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B3" s="6" t="n">
         <v>31</v>
@@ -3672,10 +3765,10 @@
         <v>5000</v>
       </c>
       <c r="N3" s="6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="O3" s="6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="P3" s="4" t="n">
         <f aca="false">ROUND(D3*C3/B3,2)+ROUND(E3*C3/B3,2)+ROUND(F3*C3/B3,2)+ROUND(G3*C3/B3,2)+H3</f>
@@ -3719,7 +3812,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B4" s="6" t="n">
         <v>28</v>
@@ -3758,10 +3851,10 @@
         <v>0</v>
       </c>
       <c r="N4" s="6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="O4" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="P4" s="4" t="n">
         <f aca="false">ROUND(D4*C4/B4,2)+ROUND(E4*C4/B4,2)+ROUND(F4*C4/B4,2)+ROUND(G4*C4/B4,2)+H4</f>
@@ -3805,7 +3898,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B5" s="6" t="n">
         <v>31</v>
@@ -3844,10 +3937,10 @@
         <v>0</v>
       </c>
       <c r="N5" s="6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="O5" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="P5" s="4" t="n">
         <f aca="false">ROUND(D5*C5/B5,2)+ROUND(E5*C5/B5,2)+ROUND(F5*C5/B5,2)+ROUND(G5*C5/B5,2)+H5</f>
@@ -3891,7 +3984,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B6" s="6" t="n">
         <v>31</v>
@@ -3930,10 +4023,10 @@
         <v>0</v>
       </c>
       <c r="N6" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="O6" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="P6" s="4" t="n">
         <f aca="false">ROUND(D6*C6/B6,2)+ROUND(E6*C6/B6,2)+ROUND(F6*C6/B6,2)+ROUND(G6*C6/B6,2)+H6</f>
@@ -3977,7 +4070,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B7" s="6" t="n">
         <v>31</v>
@@ -4016,10 +4109,10 @@
         <v>2.22</v>
       </c>
       <c r="N7" s="6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="O7" s="6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="P7" s="4" t="n">
         <f aca="false">ROUND(D7*C7/B7,2)+ROUND(E7*C7/B7,2)+ROUND(F7*C7/B7,2)+ROUND(G7*C7/B7,2)+H7</f>
@@ -4072,4 +4165,355 @@
   </headerFooter>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:R9"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="2" style="0" width="25"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>158</v>
+      </c>
+      <c r="B2" s="9" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="C2" s="9" t="n">
+        <v>90000</v>
+      </c>
+      <c r="D2" s="9" t="n">
+        <v>144000</v>
+      </c>
+      <c r="E2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="9" t="n">
+        <v>200000</v>
+      </c>
+      <c r="K2" s="4" t="n">
+        <f aca="false">B2+F2</f>
+        <v>1800000</v>
+      </c>
+      <c r="L2" s="4" t="n">
+        <f aca="false">C2+G2</f>
+        <v>90000</v>
+      </c>
+      <c r="M2" s="4" t="n">
+        <f aca="false">SUM(C2:E2)+SUM(G2:I2)</f>
+        <v>234000</v>
+      </c>
+      <c r="N2" s="4" t="n">
+        <f aca="false">K2-M2</f>
+        <v>1566000</v>
+      </c>
+      <c r="O2" s="4" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="P2" s="4" t="n">
+        <v>1566000</v>
+      </c>
+      <c r="Q2" s="4" t="n">
+        <f aca="false">K2-O2</f>
+        <v>0</v>
+      </c>
+      <c r="R2" s="4" t="n">
+        <f aca="false">N2-P2</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
+        <v>159</v>
+      </c>
+      <c r="B3" s="9" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="C3" s="9" t="n">
+        <v>90000</v>
+      </c>
+      <c r="D3" s="9" t="n">
+        <v>144000</v>
+      </c>
+      <c r="E3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="9" t="n">
+        <v>200000</v>
+      </c>
+      <c r="G3" s="9" t="n">
+        <v>17600</v>
+      </c>
+      <c r="H3" s="9" t="n">
+        <v>16000</v>
+      </c>
+      <c r="I3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="4" t="n">
+        <f aca="false">B3+F3</f>
+        <v>2000000</v>
+      </c>
+      <c r="L3" s="4" t="n">
+        <f aca="false">C3+G3</f>
+        <v>107600</v>
+      </c>
+      <c r="M3" s="4" t="n">
+        <f aca="false">SUM(C3:E3)+SUM(G3:I3)</f>
+        <v>267600</v>
+      </c>
+      <c r="N3" s="4" t="n">
+        <f aca="false">K3-M3</f>
+        <v>1732400</v>
+      </c>
+      <c r="O3" s="4" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="P3" s="4" t="n">
+        <v>1732400</v>
+      </c>
+      <c r="Q3" s="4" t="n">
+        <f aca="false">K3-O3</f>
+        <v>0</v>
+      </c>
+      <c r="R3" s="4" t="n">
+        <f aca="false">N3-P3</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="s">
+        <v>160</v>
+      </c>
+      <c r="B4" s="9" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="C4" s="9" t="n">
+        <v>90000</v>
+      </c>
+      <c r="D4" s="9" t="n">
+        <v>144000</v>
+      </c>
+      <c r="E4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="9" t="n">
+        <v>200000</v>
+      </c>
+      <c r="G4" s="9" t="n">
+        <v>17600</v>
+      </c>
+      <c r="H4" s="9" t="n">
+        <v>16000</v>
+      </c>
+      <c r="I4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="9" t="n">
+        <v>200000</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <f aca="false">B4+F4</f>
+        <v>2000000</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <f aca="false">C4+G4</f>
+        <v>107600</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <f aca="false">SUM(C4:E4)+SUM(G4:I4)</f>
+        <v>267600</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <f aca="false">K4-M4</f>
+        <v>1732400</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>1732400</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <f aca="false">K4-O4</f>
+        <v>0</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <f aca="false">N4-P4</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
+        <v>161</v>
+      </c>
+      <c r="B5" s="9" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>90000</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>144000</v>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>400000</v>
+      </c>
+      <c r="G5" s="9" t="n">
+        <v>35200</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>32000</v>
+      </c>
+      <c r="I5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="4" t="n">
+        <f aca="false">B5+F5</f>
+        <v>2200000</v>
+      </c>
+      <c r="L5" s="4" t="n">
+        <f aca="false">C5+G5</f>
+        <v>125200</v>
+      </c>
+      <c r="M5" s="4" t="n">
+        <f aca="false">SUM(C5:E5)+SUM(G5:I5)</f>
+        <v>301200</v>
+      </c>
+      <c r="N5" s="4" t="n">
+        <f aca="false">K5-M5</f>
+        <v>1898800</v>
+      </c>
+      <c r="O5" s="4" t="n">
+        <v>2200000</v>
+      </c>
+      <c r="P5" s="4" t="n">
+        <v>1898800</v>
+      </c>
+      <c r="Q5" s="4" t="n">
+        <f aca="false">K5-O5</f>
+        <v>0</v>
+      </c>
+      <c r="R5" s="4" t="n">
+        <f aca="false">N5-P5</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
+        <v>162</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="s">
+        <v>164</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="s">
+        <v>166</v>
+      </c>
+      <c r="B9" s="0" t="s">
+        <v>167</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add opt-in cumulative PAYE with authoritative history and review workbook
</commit_message>
<xml_diff>
--- a/public/payroll-review.xlsx
+++ b/public/payroll-review.xlsx
@@ -15,9 +15,11 @@
     <sheet name="Sources" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Period review" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="YTD reconciliation" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Cumulative PAYE" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Calculation!$A$1:$AA$16</definedName>
+    <definedName function="false" hidden="true" localSheetId="7" name="_xlnm._FilterDatabase" vbProcedure="false">'Cumulative PAYE'!$A$1:$Z$12</definedName>
     <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">'Period review'!$A$1:$Y$7</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -30,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="209">
   <si>
     <t xml:space="preserve">Nigeria 2026 payroll calculation review</t>
   </si>
@@ -98,7 +100,13 @@
     <t xml:space="preserve">Not supported</t>
   </si>
   <si>
-    <t xml:space="preserve">Automatic cumulative/YTD PAYE, arrears, leaver calculations, unpaid absence, foreign currency or nonresident cases.</t>
+    <t xml:space="preserve">Arrears, automatic tax refunds, leaver-specific tax, unpaid absence, foreign currency or nonresident cases.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cumulative mode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Explicit calendar-month YTD method with complete-history and evidence confirmation. See Cumulative PAYE sheet for assumptions; accountant approval remains pending.</t>
   </si>
   <si>
     <t xml:space="preserve">Sources</t>
@@ -401,6 +409,15 @@
     <t xml:space="preserve">Eligibility and 1% annual payroll contribution.</t>
   </si>
   <si>
+    <t xml:space="preserve">JRB PIT Guidelines 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://irs.kg.gov.ng/JRB_2026_PIT_Guidelines_Final.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sections 7–9, 13 and Appendix 1: cumulative records, eligible deductions, rent relief, non-periodic payments and 2026 bands. Calendar-month apportionment is an explicit implementation assumption.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Calendar days</t>
   </si>
   <si>
@@ -534,6 +551,114 @@
   </si>
   <si>
     <t xml:space="preserve">Opening references and change history are company-admin only. Released payroll review records include a calculation SHA-256 fingerprint.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calendar month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prior gross</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prior pension</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prior NHF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prior NHIS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prior PAYE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Current gross</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Current pension</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Current NHF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Current NHIS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Current other deductions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other annual reliefs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Min wage exempt?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annual rent relief</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annualised taxable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cumulative tax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Current PAYE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total current deductions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Current net</t>
+  </si>
+  <si>
+    <t xml:space="preserve">January standard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">October standard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bonus added once</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salary increase</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pension NHF rent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First job October starter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">December annual reconciliation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">December top band</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kobo rounding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmed minimum wage exemption</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prior under-deduction recovered</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Method assumption</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calendar-month YTD annualisation with proportional annual reliefs/bands. The JRB source requires cumulative records but does not prescribe this formula verbatim. Confirm method with the relevant accountant/tax authority.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eligibility</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All prior months must be covered. Eligible pension/NHF/NHIS contributions and evidence must be reviewed. Minimum-wage exemption requires explicit evidence confirmation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blocked cases</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Negative current tax indicates a possible refund; negative net indicates excessive recovery. App preview flags these and blocks automatic drafting. Workbook does not perform refunds.</t>
   </si>
 </sst>
 </file>
@@ -821,6 +946,10 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
@@ -1001,7 +1130,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
@@ -1140,6 +1269,14 @@
       </c>
       <c r="B17" s="2" t="s">
         <v>32</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -1167,15 +1304,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B2" s="3" t="n">
         <v>0.08</v>
@@ -1183,7 +1320,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B3" s="3" t="n">
         <v>0.1</v>
@@ -1191,7 +1328,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B4" s="3" t="n">
         <v>0.025</v>
@@ -1199,15 +1336,15 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B6" s="3" t="n">
         <v>0.2</v>
@@ -1215,7 +1352,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B7" s="4" t="n">
         <v>500000</v>
@@ -1231,7 +1368,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B9" s="3" t="n">
         <v>0.01</v>
@@ -1239,7 +1376,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B10" s="3" t="n">
         <v>0</v>
@@ -1247,10 +1384,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -1278,85 +1415,85 @@
   <sheetData>
     <row r="1" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>9</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="O1" s="1" t="s">
         <v>11</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1388,10 +1525,10 @@
         <v>0</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="L2" s="7" t="n">
         <f aca="false">SUM(B2:E2)</f>
@@ -1458,7 +1595,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B3" s="5" t="n">
         <v>70000.01</v>
@@ -1485,10 +1622,10 @@
         <v>0</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="L3" s="7" t="n">
         <f aca="false">SUM(B3:E3)</f>
@@ -1555,7 +1692,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B4" s="5" t="n">
         <v>200000</v>
@@ -1582,10 +1719,10 @@
         <v>0</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="L4" s="7" t="n">
         <f aca="false">SUM(B4:E4)</f>
@@ -1652,7 +1789,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B5" s="5" t="n">
         <v>250000</v>
@@ -1679,10 +1816,10 @@
         <v>0</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="L5" s="7" t="n">
         <f aca="false">SUM(B5:E5)</f>
@@ -1749,7 +1886,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B6" s="5" t="n">
         <v>1000000</v>
@@ -1776,10 +1913,10 @@
         <v>0</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="L6" s="7" t="n">
         <f aca="false">SUM(B6:E6)</f>
@@ -1846,7 +1983,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B7" s="5" t="n">
         <v>2083333.33</v>
@@ -1873,10 +2010,10 @@
         <v>0</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="L7" s="7" t="n">
         <f aca="false">SUM(B7:E7)</f>
@@ -1943,7 +2080,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B8" s="5" t="n">
         <v>4166666.67</v>
@@ -1970,10 +2107,10 @@
         <v>0</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="L8" s="7" t="n">
         <f aca="false">SUM(B8:E8)</f>
@@ -2040,7 +2177,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B9" s="5" t="n">
         <v>5000000</v>
@@ -2067,10 +2204,10 @@
         <v>0</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="L9" s="7" t="n">
         <f aca="false">SUM(B9:E9)</f>
@@ -2137,7 +2274,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B10" s="5" t="n">
         <v>200000</v>
@@ -2164,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="L10" s="7" t="n">
         <f aca="false">SUM(B10:E10)</f>
@@ -2234,7 +2371,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B11" s="5" t="n">
         <v>350000</v>
@@ -2261,10 +2398,10 @@
         <v>0</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="L11" s="7" t="n">
         <f aca="false">SUM(B11:E11)</f>
@@ -2331,7 +2468,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B12" s="5" t="n">
         <v>250000</v>
@@ -2358,10 +2495,10 @@
         <v>0</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="K12" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="L12" s="7" t="n">
         <f aca="false">SUM(B12:E12)</f>
@@ -2428,7 +2565,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B13" s="5" t="n">
         <v>200000</v>
@@ -2455,10 +2592,10 @@
         <v>0</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="L13" s="7" t="n">
         <f aca="false">SUM(B13:E13)</f>
@@ -2525,7 +2662,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B14" s="5" t="n">
         <v>200000</v>
@@ -2552,10 +2689,10 @@
         <v>120000</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="K14" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="L14" s="7" t="n">
         <f aca="false">SUM(B14:E14)</f>
@@ -2622,7 +2759,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B15" s="5" t="n">
         <v>123456.78</v>
@@ -2649,10 +2786,10 @@
         <v>0</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="L15" s="7" t="n">
         <f aca="false">SUM(B15:E15)</f>
@@ -2719,7 +2856,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B16" s="5" t="n">
         <v>100000</v>
@@ -2746,10 +2883,10 @@
         <v>1200000</v>
       </c>
       <c r="J16" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="K16" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="L16" s="7" t="n">
         <f aca="false">SUM(B16:E16)</f>
@@ -2847,37 +2984,37 @@
   <sheetData>
     <row r="1" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2917,7 +3054,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B3" s="0" t="n">
         <v>70000.01</v>
@@ -2952,7 +3089,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B4" s="0" t="n">
         <v>200000</v>
@@ -2987,7 +3124,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B5" s="0" t="n">
         <v>250000</v>
@@ -3022,7 +3159,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B6" s="0" t="n">
         <v>1000000</v>
@@ -3057,7 +3194,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B7" s="0" t="n">
         <v>2083333.33</v>
@@ -3092,7 +3229,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B8" s="0" t="n">
         <v>4166666.67</v>
@@ -3127,7 +3264,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B9" s="0" t="n">
         <v>5000000</v>
@@ -3162,7 +3299,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B10" s="0" t="n">
         <v>350000</v>
@@ -3197,7 +3334,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B11" s="0" t="n">
         <v>350000</v>
@@ -3232,7 +3369,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B12" s="0" t="n">
         <v>250000</v>
@@ -3267,7 +3404,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B13" s="0" t="n">
         <v>350000</v>
@@ -3302,7 +3439,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B14" s="0" t="n">
         <v>200000</v>
@@ -3337,7 +3474,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B15" s="0" t="n">
         <v>150370.35</v>
@@ -3372,7 +3509,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B16" s="0" t="n">
         <v>100000</v>
@@ -3421,7 +3558,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
@@ -3431,101 +3568,112 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>122</v>
+        <v>124</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="s">
+        <v>125</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="C10" s="0" t="s">
+        <v>127</v>
       </c>
     </row>
   </sheetData>
@@ -3538,6 +3686,7 @@
     <hyperlink ref="B7" r:id="rId6" display="https://www.fmbn.gov.ng/documents/FMBN_SERVICOM_CHARTER.pdf"/>
     <hyperlink ref="B8" r:id="rId7" display="https://nsitf.gov.ng/services"/>
     <hyperlink ref="B9" r:id="rId8" display="https://www.itf.gov.ng/"/>
+    <hyperlink ref="B10" r:id="rId9" display="https://irs.kg.gov.ng/JRB_2026_PIT_Guidelines_Final.pdf"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3563,84 +3712,84 @@
   <sheetData>
     <row r="1" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="S1" s="1" t="s">
         <v>11</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="B2" s="6" t="n">
         <v>31</v>
@@ -3679,10 +3828,10 @@
         <v>5000</v>
       </c>
       <c r="N2" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="O2" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="P2" s="4" t="n">
         <f aca="false">ROUND(D2*C2/B2,2)+ROUND(E2*C2/B2,2)+ROUND(F2*C2/B2,2)+ROUND(G2*C2/B2,2)+H2</f>
@@ -3726,7 +3875,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="B3" s="6" t="n">
         <v>31</v>
@@ -3765,10 +3914,10 @@
         <v>5000</v>
       </c>
       <c r="N3" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="O3" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="P3" s="4" t="n">
         <f aca="false">ROUND(D3*C3/B3,2)+ROUND(E3*C3/B3,2)+ROUND(F3*C3/B3,2)+ROUND(G3*C3/B3,2)+H3</f>
@@ -3812,7 +3961,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="B4" s="6" t="n">
         <v>28</v>
@@ -3851,10 +4000,10 @@
         <v>0</v>
       </c>
       <c r="N4" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="O4" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="P4" s="4" t="n">
         <f aca="false">ROUND(D4*C4/B4,2)+ROUND(E4*C4/B4,2)+ROUND(F4*C4/B4,2)+ROUND(G4*C4/B4,2)+H4</f>
@@ -3898,7 +4047,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="B5" s="6" t="n">
         <v>31</v>
@@ -3937,10 +4086,10 @@
         <v>0</v>
       </c>
       <c r="N5" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="O5" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="P5" s="4" t="n">
         <f aca="false">ROUND(D5*C5/B5,2)+ROUND(E5*C5/B5,2)+ROUND(F5*C5/B5,2)+ROUND(G5*C5/B5,2)+H5</f>
@@ -3984,7 +4133,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="B6" s="6" t="n">
         <v>31</v>
@@ -4023,10 +4172,10 @@
         <v>0</v>
       </c>
       <c r="N6" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="O6" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="P6" s="4" t="n">
         <f aca="false">ROUND(D6*C6/B6,2)+ROUND(E6*C6/B6,2)+ROUND(F6*C6/B6,2)+ROUND(G6*C6/B6,2)+H6</f>
@@ -4070,7 +4219,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="B7" s="6" t="n">
         <v>31</v>
@@ -4109,10 +4258,10 @@
         <v>2.22</v>
       </c>
       <c r="N7" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="O7" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="P7" s="4" t="n">
         <f aca="false">ROUND(D7*C7/B7,2)+ROUND(E7*C7/B7,2)+ROUND(F7*C7/B7,2)+ROUND(G7*C7/B7,2)+H7</f>
@@ -4181,63 +4330,63 @@
   <sheetData>
     <row r="1" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="B2" s="9" t="n">
         <v>1800000</v>
@@ -4299,7 +4448,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="B3" s="9" t="n">
         <v>1800000</v>
@@ -4361,7 +4510,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="B4" s="9" t="n">
         <v>1800000</v>
@@ -4423,7 +4572,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="B5" s="9" t="n">
         <v>1800000</v>
@@ -4485,26 +4634,26 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
     </row>
   </sheetData>
@@ -4516,4 +4665,1112 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:Z16"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="2" style="0" width="23"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>192</v>
+      </c>
+      <c r="B2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="9" t="n">
+        <v>200000</v>
+      </c>
+      <c r="I2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="P2" s="4" t="n">
+        <f aca="false">MIN(ROUND(M2*0.2,2),500000)</f>
+        <v>0</v>
+      </c>
+      <c r="Q2" s="4" t="n">
+        <f aca="false">MAX(0,(C2+H2-D2-I2-E2-J2-F2-K2)*12/B2-P2-N2)</f>
+        <v>2400000</v>
+      </c>
+      <c r="R2" s="4" t="n">
+        <f aca="false">MIN(MAX(Q2-800000,0),2200000)*0.15+MIN(MAX(Q2-3000000,0),9000000)*0.18+MIN(MAX(Q2-12000000,0),13000000)*0.21+MIN(MAX(Q2-25000000,0),25000000)*0.23+MAX(Q2-50000000,0)*0.25</f>
+        <v>240000</v>
+      </c>
+      <c r="S2" s="4" t="n">
+        <f aca="false">IF(O2="Yes",0,ROUND(R2*B2/12,2))</f>
+        <v>20000</v>
+      </c>
+      <c r="T2" s="4" t="n">
+        <f aca="false">MAX(0,S2-G2)</f>
+        <v>20000</v>
+      </c>
+      <c r="U2" s="4" t="n">
+        <f aca="false">SUM(I2:L2)+T2</f>
+        <v>20000</v>
+      </c>
+      <c r="V2" s="4" t="n">
+        <f aca="false">H2-U2</f>
+        <v>180000</v>
+      </c>
+      <c r="W2" s="4" t="n">
+        <v>20000</v>
+      </c>
+      <c r="X2" s="4" t="n">
+        <v>180000</v>
+      </c>
+      <c r="Y2" s="4" t="n">
+        <f aca="false">T2-W2</f>
+        <v>0</v>
+      </c>
+      <c r="Z2" s="4" t="n">
+        <f aca="false">V2-X2</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
+        <v>193</v>
+      </c>
+      <c r="B3" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="C3" s="9" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="D3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="9" t="n">
+        <v>180000</v>
+      </c>
+      <c r="H3" s="9" t="n">
+        <v>200000</v>
+      </c>
+      <c r="I3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="P3" s="4" t="n">
+        <f aca="false">MIN(ROUND(M3*0.2,2),500000)</f>
+        <v>0</v>
+      </c>
+      <c r="Q3" s="4" t="n">
+        <f aca="false">MAX(0,(C3+H3-D3-I3-E3-J3-F3-K3)*12/B3-P3-N3)</f>
+        <v>2400000</v>
+      </c>
+      <c r="R3" s="4" t="n">
+        <f aca="false">MIN(MAX(Q3-800000,0),2200000)*0.15+MIN(MAX(Q3-3000000,0),9000000)*0.18+MIN(MAX(Q3-12000000,0),13000000)*0.21+MIN(MAX(Q3-25000000,0),25000000)*0.23+MAX(Q3-50000000,0)*0.25</f>
+        <v>240000</v>
+      </c>
+      <c r="S3" s="4" t="n">
+        <f aca="false">IF(O3="Yes",0,ROUND(R3*B3/12,2))</f>
+        <v>200000</v>
+      </c>
+      <c r="T3" s="4" t="n">
+        <f aca="false">MAX(0,S3-G3)</f>
+        <v>20000</v>
+      </c>
+      <c r="U3" s="4" t="n">
+        <f aca="false">SUM(I3:L3)+T3</f>
+        <v>20000</v>
+      </c>
+      <c r="V3" s="4" t="n">
+        <f aca="false">H3-U3</f>
+        <v>180000</v>
+      </c>
+      <c r="W3" s="4" t="n">
+        <v>20000</v>
+      </c>
+      <c r="X3" s="4" t="n">
+        <v>180000</v>
+      </c>
+      <c r="Y3" s="4" t="n">
+        <f aca="false">T3-W3</f>
+        <v>0</v>
+      </c>
+      <c r="Z3" s="4" t="n">
+        <f aca="false">V3-X3</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="s">
+        <v>194</v>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="C4" s="9" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="D4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="9" t="n">
+        <v>180000</v>
+      </c>
+      <c r="H4" s="9" t="n">
+        <v>300000</v>
+      </c>
+      <c r="I4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <f aca="false">MIN(ROUND(M4*0.2,2),500000)</f>
+        <v>0</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <f aca="false">MAX(0,(C4+H4-D4-I4-E4-J4-F4-K4)*12/B4-P4-N4)</f>
+        <v>2520000</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <f aca="false">MIN(MAX(Q4-800000,0),2200000)*0.15+MIN(MAX(Q4-3000000,0),9000000)*0.18+MIN(MAX(Q4-12000000,0),13000000)*0.21+MIN(MAX(Q4-25000000,0),25000000)*0.23+MAX(Q4-50000000,0)*0.25</f>
+        <v>258000</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <f aca="false">IF(O4="Yes",0,ROUND(R4*B4/12,2))</f>
+        <v>215000</v>
+      </c>
+      <c r="T4" s="4" t="n">
+        <f aca="false">MAX(0,S4-G4)</f>
+        <v>35000</v>
+      </c>
+      <c r="U4" s="4" t="n">
+        <f aca="false">SUM(I4:L4)+T4</f>
+        <v>35000</v>
+      </c>
+      <c r="V4" s="4" t="n">
+        <f aca="false">H4-U4</f>
+        <v>265000</v>
+      </c>
+      <c r="W4" s="4" t="n">
+        <v>35000</v>
+      </c>
+      <c r="X4" s="4" t="n">
+        <v>265000</v>
+      </c>
+      <c r="Y4" s="4" t="n">
+        <f aca="false">T4-W4</f>
+        <v>0</v>
+      </c>
+      <c r="Z4" s="4" t="n">
+        <f aca="false">V4-X4</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
+        <v>195</v>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="9" t="n">
+        <v>180000</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>300000</v>
+      </c>
+      <c r="I5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="P5" s="4" t="n">
+        <f aca="false">MIN(ROUND(M5*0.2,2),500000)</f>
+        <v>0</v>
+      </c>
+      <c r="Q5" s="4" t="n">
+        <f aca="false">MAX(0,(C5+H5-D5-I5-E5-J5-F5-K5)*12/B5-P5-N5)</f>
+        <v>2520000</v>
+      </c>
+      <c r="R5" s="4" t="n">
+        <f aca="false">MIN(MAX(Q5-800000,0),2200000)*0.15+MIN(MAX(Q5-3000000,0),9000000)*0.18+MIN(MAX(Q5-12000000,0),13000000)*0.21+MIN(MAX(Q5-25000000,0),25000000)*0.23+MAX(Q5-50000000,0)*0.25</f>
+        <v>258000</v>
+      </c>
+      <c r="S5" s="4" t="n">
+        <f aca="false">IF(O5="Yes",0,ROUND(R5*B5/12,2))</f>
+        <v>215000</v>
+      </c>
+      <c r="T5" s="4" t="n">
+        <f aca="false">MAX(0,S5-G5)</f>
+        <v>35000</v>
+      </c>
+      <c r="U5" s="4" t="n">
+        <f aca="false">SUM(I5:L5)+T5</f>
+        <v>35000</v>
+      </c>
+      <c r="V5" s="4" t="n">
+        <f aca="false">H5-U5</f>
+        <v>265000</v>
+      </c>
+      <c r="W5" s="4" t="n">
+        <v>35000</v>
+      </c>
+      <c r="X5" s="4" t="n">
+        <v>265000</v>
+      </c>
+      <c r="Y5" s="4" t="n">
+        <f aca="false">T5-W5</f>
+        <v>0</v>
+      </c>
+      <c r="Z5" s="4" t="n">
+        <f aca="false">V5-X5</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="s">
+        <v>196</v>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>3150000</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>252000</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>45000</v>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="9" t="n">
+        <v>323640</v>
+      </c>
+      <c r="H6" s="9" t="n">
+        <v>350000</v>
+      </c>
+      <c r="I6" s="9" t="n">
+        <v>28000</v>
+      </c>
+      <c r="J6" s="9" t="n">
+        <v>5000</v>
+      </c>
+      <c r="K6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="9" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="N6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <f aca="false">MIN(ROUND(M6*0.2,2),500000)</f>
+        <v>240000</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <f aca="false">MAX(0,(C6+H6-D6-I6-E6-J6-F6-K6)*12/B6-P6-N6)</f>
+        <v>3564000</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <f aca="false">MIN(MAX(Q6-800000,0),2200000)*0.15+MIN(MAX(Q6-3000000,0),9000000)*0.18+MIN(MAX(Q6-12000000,0),13000000)*0.21+MIN(MAX(Q6-25000000,0),25000000)*0.23+MAX(Q6-50000000,0)*0.25</f>
+        <v>431520</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <f aca="false">IF(O6="Yes",0,ROUND(R6*B6/12,2))</f>
+        <v>359600</v>
+      </c>
+      <c r="T6" s="4" t="n">
+        <f aca="false">MAX(0,S6-G6)</f>
+        <v>35960</v>
+      </c>
+      <c r="U6" s="4" t="n">
+        <f aca="false">SUM(I6:L6)+T6</f>
+        <v>68960</v>
+      </c>
+      <c r="V6" s="4" t="n">
+        <f aca="false">H6-U6</f>
+        <v>281040</v>
+      </c>
+      <c r="W6" s="4" t="n">
+        <v>35960</v>
+      </c>
+      <c r="X6" s="4" t="n">
+        <v>281040</v>
+      </c>
+      <c r="Y6" s="4" t="n">
+        <f aca="false">T6-W6</f>
+        <v>0</v>
+      </c>
+      <c r="Z6" s="4" t="n">
+        <f aca="false">V6-X6</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
+        <v>197</v>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="9" t="n">
+        <v>160000</v>
+      </c>
+      <c r="I7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="P7" s="4" t="n">
+        <f aca="false">MIN(ROUND(M7*0.2,2),500000)</f>
+        <v>0</v>
+      </c>
+      <c r="Q7" s="4" t="n">
+        <f aca="false">MAX(0,(C7+H7-D7-I7-E7-J7-F7-K7)*12/B7-P7-N7)</f>
+        <v>192000</v>
+      </c>
+      <c r="R7" s="4" t="n">
+        <f aca="false">MIN(MAX(Q7-800000,0),2200000)*0.15+MIN(MAX(Q7-3000000,0),9000000)*0.18+MIN(MAX(Q7-12000000,0),13000000)*0.21+MIN(MAX(Q7-25000000,0),25000000)*0.23+MAX(Q7-50000000,0)*0.25</f>
+        <v>0</v>
+      </c>
+      <c r="S7" s="4" t="n">
+        <f aca="false">IF(O7="Yes",0,ROUND(R7*B7/12,2))</f>
+        <v>0</v>
+      </c>
+      <c r="T7" s="4" t="n">
+        <f aca="false">MAX(0,S7-G7)</f>
+        <v>0</v>
+      </c>
+      <c r="U7" s="4" t="n">
+        <f aca="false">SUM(I7:L7)+T7</f>
+        <v>0</v>
+      </c>
+      <c r="V7" s="4" t="n">
+        <f aca="false">H7-U7</f>
+        <v>160000</v>
+      </c>
+      <c r="W7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X7" s="4" t="n">
+        <v>160000</v>
+      </c>
+      <c r="Y7" s="4" t="n">
+        <f aca="false">T7-W7</f>
+        <v>0</v>
+      </c>
+      <c r="Z7" s="4" t="n">
+        <f aca="false">V7-X7</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="s">
+        <v>198</v>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>2750000</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="9" t="n">
+        <v>302500</v>
+      </c>
+      <c r="H8" s="9" t="n">
+        <v>250000</v>
+      </c>
+      <c r="I8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <f aca="false">MIN(ROUND(M8*0.2,2),500000)</f>
+        <v>0</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <f aca="false">MAX(0,(C8+H8-D8-I8-E8-J8-F8-K8)*12/B8-P8-N8)</f>
+        <v>3000000</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <f aca="false">MIN(MAX(Q8-800000,0),2200000)*0.15+MIN(MAX(Q8-3000000,0),9000000)*0.18+MIN(MAX(Q8-12000000,0),13000000)*0.21+MIN(MAX(Q8-25000000,0),25000000)*0.23+MAX(Q8-50000000,0)*0.25</f>
+        <v>330000</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <f aca="false">IF(O8="Yes",0,ROUND(R8*B8/12,2))</f>
+        <v>330000</v>
+      </c>
+      <c r="T8" s="4" t="n">
+        <f aca="false">MAX(0,S8-G8)</f>
+        <v>27500</v>
+      </c>
+      <c r="U8" s="4" t="n">
+        <f aca="false">SUM(I8:L8)+T8</f>
+        <v>27500</v>
+      </c>
+      <c r="V8" s="4" t="n">
+        <f aca="false">H8-U8</f>
+        <v>222500</v>
+      </c>
+      <c r="W8" s="4" t="n">
+        <v>27500</v>
+      </c>
+      <c r="X8" s="4" t="n">
+        <v>222500</v>
+      </c>
+      <c r="Y8" s="4" t="n">
+        <f aca="false">T8-W8</f>
+        <v>0</v>
+      </c>
+      <c r="Z8" s="4" t="n">
+        <f aca="false">V8-X8</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="s">
+        <v>199</v>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="C9" s="9" t="n">
+        <v>55000000</v>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="9" t="n">
+        <v>11852500</v>
+      </c>
+      <c r="H9" s="9" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="I9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="P9" s="4" t="n">
+        <f aca="false">MIN(ROUND(M9*0.2,2),500000)</f>
+        <v>0</v>
+      </c>
+      <c r="Q9" s="4" t="n">
+        <f aca="false">MAX(0,(C9+H9-D9-I9-E9-J9-F9-K9)*12/B9-P9-N9)</f>
+        <v>60000000</v>
+      </c>
+      <c r="R9" s="4" t="n">
+        <f aca="false">MIN(MAX(Q9-800000,0),2200000)*0.15+MIN(MAX(Q9-3000000,0),9000000)*0.18+MIN(MAX(Q9-12000000,0),13000000)*0.21+MIN(MAX(Q9-25000000,0),25000000)*0.23+MAX(Q9-50000000,0)*0.25</f>
+        <v>12930000</v>
+      </c>
+      <c r="S9" s="4" t="n">
+        <f aca="false">IF(O9="Yes",0,ROUND(R9*B9/12,2))</f>
+        <v>12930000</v>
+      </c>
+      <c r="T9" s="4" t="n">
+        <f aca="false">MAX(0,S9-G9)</f>
+        <v>1077500</v>
+      </c>
+      <c r="U9" s="4" t="n">
+        <f aca="false">SUM(I9:L9)+T9</f>
+        <v>1077500</v>
+      </c>
+      <c r="V9" s="4" t="n">
+        <f aca="false">H9-U9</f>
+        <v>3922500</v>
+      </c>
+      <c r="W9" s="4" t="n">
+        <v>1077500</v>
+      </c>
+      <c r="X9" s="4" t="n">
+        <v>3922500</v>
+      </c>
+      <c r="Y9" s="4" t="n">
+        <f aca="false">T9-W9</f>
+        <v>0</v>
+      </c>
+      <c r="Z9" s="4" t="n">
+        <f aca="false">V9-X9</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="s">
+        <v>200</v>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>1200000.06</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>96000</v>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>74.04</v>
+      </c>
+      <c r="G10" s="9" t="n">
+        <v>60000</v>
+      </c>
+      <c r="H10" s="9" t="n">
+        <v>200000.01</v>
+      </c>
+      <c r="I10" s="9" t="n">
+        <v>16000</v>
+      </c>
+      <c r="J10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="9" t="n">
+        <v>12.34</v>
+      </c>
+      <c r="L10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="9" t="n">
+        <v>987654.32</v>
+      </c>
+      <c r="N10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <f aca="false">MIN(ROUND(M10*0.2,2),500000)</f>
+        <v>197530.86</v>
+      </c>
+      <c r="Q10" s="4" t="n">
+        <f aca="false">MAX(0,(C10+H10-D10-I10-E10-J10-F10-K10)*12/B10-P10-N10)</f>
+        <v>2010321.18</v>
+      </c>
+      <c r="R10" s="4" t="n">
+        <f aca="false">MIN(MAX(Q10-800000,0),2200000)*0.15+MIN(MAX(Q10-3000000,0),9000000)*0.18+MIN(MAX(Q10-12000000,0),13000000)*0.21+MIN(MAX(Q10-25000000,0),25000000)*0.23+MAX(Q10-50000000,0)*0.25</f>
+        <v>181548.177</v>
+      </c>
+      <c r="S10" s="4" t="n">
+        <f aca="false">IF(O10="Yes",0,ROUND(R10*B10/12,2))</f>
+        <v>105903.1</v>
+      </c>
+      <c r="T10" s="4" t="n">
+        <f aca="false">MAX(0,S10-G10)</f>
+        <v>45903.1</v>
+      </c>
+      <c r="U10" s="4" t="n">
+        <f aca="false">SUM(I10:L10)+T10</f>
+        <v>61915.44</v>
+      </c>
+      <c r="V10" s="4" t="n">
+        <f aca="false">H10-U10</f>
+        <v>138084.57</v>
+      </c>
+      <c r="W10" s="4" t="n">
+        <v>45903.1</v>
+      </c>
+      <c r="X10" s="4" t="n">
+        <v>138084.57</v>
+      </c>
+      <c r="Y10" s="4" t="n">
+        <f aca="false">T10-W10</f>
+        <v>0</v>
+      </c>
+      <c r="Z10" s="4" t="n">
+        <f aca="false">V10-X10</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="s">
+        <v>201</v>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>630000</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="9" t="n">
+        <v>70000</v>
+      </c>
+      <c r="I11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="P11" s="4" t="n">
+        <f aca="false">MIN(ROUND(M11*0.2,2),500000)</f>
+        <v>0</v>
+      </c>
+      <c r="Q11" s="4" t="n">
+        <f aca="false">MAX(0,(C11+H11-D11-I11-E11-J11-F11-K11)*12/B11-P11-N11)</f>
+        <v>840000</v>
+      </c>
+      <c r="R11" s="4" t="n">
+        <f aca="false">MIN(MAX(Q11-800000,0),2200000)*0.15+MIN(MAX(Q11-3000000,0),9000000)*0.18+MIN(MAX(Q11-12000000,0),13000000)*0.21+MIN(MAX(Q11-25000000,0),25000000)*0.23+MAX(Q11-50000000,0)*0.25</f>
+        <v>6000</v>
+      </c>
+      <c r="S11" s="4" t="n">
+        <f aca="false">IF(O11="Yes",0,ROUND(R11*B11/12,2))</f>
+        <v>0</v>
+      </c>
+      <c r="T11" s="4" t="n">
+        <f aca="false">MAX(0,S11-G11)</f>
+        <v>0</v>
+      </c>
+      <c r="U11" s="4" t="n">
+        <f aca="false">SUM(I11:L11)+T11</f>
+        <v>0</v>
+      </c>
+      <c r="V11" s="4" t="n">
+        <f aca="false">H11-U11</f>
+        <v>70000</v>
+      </c>
+      <c r="W11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X11" s="4" t="n">
+        <v>70000</v>
+      </c>
+      <c r="Y11" s="4" t="n">
+        <f aca="false">T11-W11</f>
+        <v>0</v>
+      </c>
+      <c r="Z11" s="4" t="n">
+        <f aca="false">V11-X11</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="s">
+        <v>202</v>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>144000</v>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="9" t="n">
+        <v>90000</v>
+      </c>
+      <c r="H12" s="9" t="n">
+        <v>200000</v>
+      </c>
+      <c r="I12" s="9" t="n">
+        <v>16000</v>
+      </c>
+      <c r="J12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="P12" s="4" t="n">
+        <f aca="false">MIN(ROUND(M12*0.2,2),500000)</f>
+        <v>0</v>
+      </c>
+      <c r="Q12" s="4" t="n">
+        <f aca="false">MAX(0,(C12+H12-D12-I12-E12-J12-F12-K12)*12/B12-P12-N12)</f>
+        <v>2208000</v>
+      </c>
+      <c r="R12" s="4" t="n">
+        <f aca="false">MIN(MAX(Q12-800000,0),2200000)*0.15+MIN(MAX(Q12-3000000,0),9000000)*0.18+MIN(MAX(Q12-12000000,0),13000000)*0.21+MIN(MAX(Q12-25000000,0),25000000)*0.23+MAX(Q12-50000000,0)*0.25</f>
+        <v>211200</v>
+      </c>
+      <c r="S12" s="4" t="n">
+        <f aca="false">IF(O12="Yes",0,ROUND(R12*B12/12,2))</f>
+        <v>176000</v>
+      </c>
+      <c r="T12" s="4" t="n">
+        <f aca="false">MAX(0,S12-G12)</f>
+        <v>86000</v>
+      </c>
+      <c r="U12" s="4" t="n">
+        <f aca="false">SUM(I12:L12)+T12</f>
+        <v>102000</v>
+      </c>
+      <c r="V12" s="4" t="n">
+        <f aca="false">H12-U12</f>
+        <v>98000</v>
+      </c>
+      <c r="W12" s="4" t="n">
+        <v>86000</v>
+      </c>
+      <c r="X12" s="4" t="n">
+        <v>98000</v>
+      </c>
+      <c r="Y12" s="4" t="n">
+        <f aca="false">T12-W12</f>
+        <v>0</v>
+      </c>
+      <c r="Z12" s="4" t="n">
+        <f aca="false">V12-X12</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="0" t="s">
+        <v>203</v>
+      </c>
+      <c r="B14" s="0" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="0" t="s">
+        <v>205</v>
+      </c>
+      <c r="B15" s="0" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="B16" s="0" t="s">
+        <v>208</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:Z12"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>